<commit_message>
Added new RDF data schemes and visual schemes for education-table23-28, fixed XLSX spreadsheets for education-table24-28
</commit_message>
<xml_diff>
--- a/sources/table_normalization/xlsx/education-table24.xlsx
+++ b/sources/table_normalization/xlsx/education-table24.xlsx
@@ -226,8 +226,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="2">
-    <numFmt numFmtId="168" formatCode="#,##0_)"/>
-    <numFmt numFmtId="169" formatCode="#,##0.0_)"/>
+    <numFmt numFmtId="164" formatCode="#,##0_)"/>
+    <numFmt numFmtId="165" formatCode="#,##0.0_)"/>
   </numFmts>
   <fonts count="9">
     <font>
@@ -619,64 +619,88 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="13" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="1" fillId="2" borderId="14" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="2" borderId="14" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="168" fontId="1" fillId="2" borderId="15" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="2" borderId="15" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="169" fontId="1" fillId="2" borderId="16" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="1" fillId="2" borderId="16" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="5" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="1" fillId="0" borderId="14" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="14" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="168" fontId="1" fillId="0" borderId="15" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="15" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="169" fontId="1" fillId="0" borderId="16" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="16" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="5" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="5" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="1" fillId="0" borderId="18" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="18" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="168" fontId="1" fillId="0" borderId="11" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="11" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="169" fontId="1" fillId="0" borderId="19" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="19" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="1" fillId="2" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="2" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="37" fontId="1" fillId="2" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="169" fontId="1" fillId="2" borderId="24" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="1" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="1" fillId="2" borderId="24" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="37" fontId="1" fillId="0" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="169" fontId="1" fillId="0" borderId="24" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="1" fillId="0" borderId="17" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="24" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="17" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="37" fontId="1" fillId="0" borderId="18" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="169" fontId="1" fillId="0" borderId="25" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="25" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="4" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="1" fontId="4" fillId="0" borderId="3" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="4" fillId="0" borderId="4" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="4" fillId="0" borderId="20" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="4" borderId="11" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="4" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="4" borderId="17" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="4" borderId="21" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="4" borderId="14" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="4" borderId="18" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="4" borderId="22" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="4" borderId="24" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="4" borderId="25" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="4" fillId="0" borderId="7" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -687,56 +711,32 @@
     <xf numFmtId="1" fontId="4" fillId="0" borderId="23" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="5" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="9" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="1" fontId="4" fillId="4" borderId="2" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="4" fillId="4" borderId="21" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="4" fillId="4" borderId="22" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="5" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="1" fontId="4" fillId="4" borderId="6" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="4" fillId="4" borderId="14" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="4" fillId="4" borderId="24" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="9" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="1" fontId="4" fillId="4" borderId="10" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="4" fillId="4" borderId="11" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="4" fillId="4" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="4" fillId="4" borderId="17" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="4" fillId="4" borderId="18" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="4" fillId="4" borderId="25" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="1" fontId="4" fillId="4" borderId="3" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="4" borderId="4" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="4" borderId="20" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -1091,56 +1091,56 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" s="1" customFormat="1" ht="25" customHeight="1">
-      <c r="A1" s="39" t="s">
+      <c r="A1" s="45" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="40" t="s">
+      <c r="B1" s="48" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="31" t="s">
+      <c r="C1" s="51" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
-      <c r="F1" s="33"/>
-      <c r="G1" s="41" t="s">
+      <c r="D1" s="52"/>
+      <c r="E1" s="52"/>
+      <c r="F1" s="53"/>
+      <c r="G1" s="36" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="42" t="s">
+      <c r="H1" s="39" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:10" s="1" customFormat="1" ht="25" customHeight="1">
-      <c r="A2" s="43"/>
-      <c r="B2" s="44"/>
-      <c r="C2" s="34" t="s">
+      <c r="A2" s="46"/>
+      <c r="B2" s="49"/>
+      <c r="C2" s="42" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="35"/>
-      <c r="E2" s="36" t="s">
+      <c r="D2" s="43"/>
+      <c r="E2" s="44" t="s">
         <v>6</v>
       </c>
-      <c r="F2" s="35"/>
-      <c r="G2" s="45"/>
-      <c r="H2" s="46"/>
+      <c r="F2" s="43"/>
+      <c r="G2" s="37"/>
+      <c r="H2" s="40"/>
     </row>
     <row r="3" spans="1:10" s="1" customFormat="1" ht="15" customHeight="1">
       <c r="A3" s="47"/>
-      <c r="B3" s="48"/>
-      <c r="C3" s="49" t="s">
+      <c r="B3" s="50"/>
+      <c r="C3" s="33" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="50" t="s">
+      <c r="D3" s="34" t="s">
         <v>8</v>
       </c>
-      <c r="E3" s="51" t="s">
+      <c r="E3" s="35" t="s">
         <v>7</v>
       </c>
-      <c r="F3" s="50" t="s">
+      <c r="F3" s="34" t="s">
         <v>8</v>
       </c>
-      <c r="G3" s="52"/>
-      <c r="H3" s="53"/>
+      <c r="G3" s="38"/>
+      <c r="H3" s="41"/>
     </row>
     <row r="4" spans="1:10" s="2" customFormat="1" ht="15" customHeight="1">
       <c r="A4" s="6" t="s">
@@ -2518,7 +2518,7 @@
       <c r="T56" s="19"/>
     </row>
     <row r="57" spans="1:22" s="3" customFormat="1" ht="15" customHeight="1">
-      <c r="A57" s="37" t="str">
+      <c r="A57" s="31" t="str">
         <f>CONCATENATE("NOTE: Table reads (for US Totals):  Of all ",IF(ISTEXT(B4),LEFT(B4,3),TEXT(B4,"#,##0"))," public schools with grades 7 and 8, ",IF(ISTEXT(C4),LEFT(C4,3),TEXT(C4,"#,##0"))," (",TEXT(D4,"0.0"),"%) offered Algebra I classes.")</f>
         <v>NOTE: Table reads (for US Totals):  Of all 30,650 public schools with grades 7 and 8, 18,258 (59.6%) offered Algebra I classes.</v>
       </c>
@@ -2543,7 +2543,7 @@
       <c r="T57" s="19"/>
     </row>
     <row r="58" spans="1:22" s="3" customFormat="1" ht="14.15" customHeight="1">
-      <c r="A58" s="38" t="s">
+      <c r="A58" s="32" t="s">
         <v>61</v>
       </c>
       <c r="B58" s="20"/>
@@ -2569,7 +2569,7 @@
       <c r="V58" s="20"/>
     </row>
     <row r="59" spans="1:22" s="3" customFormat="1" ht="15" customHeight="1">
-      <c r="A59" s="38" t="s">
+      <c r="A59" s="32" t="s">
         <v>62</v>
       </c>
       <c r="B59" s="20"/>
@@ -2599,13 +2599,13 @@
     <sortCondition ref="A8:A58"/>
   </sortState>
   <mergeCells count="7">
+    <mergeCell ref="A1:A3"/>
+    <mergeCell ref="B1:B3"/>
     <mergeCell ref="G1:G3"/>
     <mergeCell ref="H1:H3"/>
     <mergeCell ref="C1:F1"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="E2:F2"/>
-    <mergeCell ref="A1:A3"/>
-    <mergeCell ref="B1:B3"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.5" right="0.5" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>